<commit_message>
Build site at 2021-05-18 16:02:34 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
+++ b/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="208">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -560,6 +560,81 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1NOr-z6RTE9-w0_Zl-yNqVx1YerdXTO4Q</t>
+  </si>
+  <si>
+    <t>Rafaela dos Santos Silva</t>
+  </si>
+  <si>
+    <t>rafaelasantos@id.uff.br</t>
+  </si>
+  <si>
+    <t>Feminino</t>
+  </si>
+  <si>
+    <t>Solteiro (a)</t>
+  </si>
+  <si>
+    <t>Parda</t>
+  </si>
+  <si>
+    <t>Volta Redonda</t>
+  </si>
+  <si>
+    <t>Brasil</t>
+  </si>
+  <si>
+    <t>Detran</t>
+  </si>
+  <si>
+    <t>Rua Quinhentos e Quarenta e Oito, 249</t>
+  </si>
+  <si>
+    <t>Jardim Paraíba</t>
+  </si>
+  <si>
+    <t>Celular</t>
+  </si>
+  <si>
+    <t>Vera Lúcia dos Santos</t>
+  </si>
+  <si>
+    <t>Mãe</t>
+  </si>
+  <si>
+    <t>Rio de Janeiro/Brasil</t>
+  </si>
+  <si>
+    <t>Universidade Federal Fluminense</t>
+  </si>
+  <si>
+    <t>Mestrado Em Engenharia Metalúrgica</t>
+  </si>
+  <si>
+    <t>Graduação em Engenharia Metalúrgica</t>
+  </si>
+  <si>
+    <t>Instituto Federal de Educação, Ciência e Tecnologia do Rio de Janeiro</t>
+  </si>
+  <si>
+    <t>Técnica em Automação Industrial</t>
+  </si>
+  <si>
+    <t>Estágio à docência</t>
+  </si>
+  <si>
+    <t>Continuar a trabalhar com pesquisa na área de materiais metálicos e aprender a prática de ensino da engenharia.</t>
+  </si>
+  <si>
+    <t>Aluno PPGEM</t>
+  </si>
+  <si>
+    <t>Análise do comportamento em fluência e de oxidação da superliga MAR-M247 modificada com Nb e produzida por solidificação direcional</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=13RWTnMFln-Or9zzfvdd5gCUDLWq4PLXD</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1h66cbUGy55OyDA-DH5yFT0ZNjRLK4dS9</t>
   </si>
 </sst>
 </file>
@@ -1825,12 +1900,231 @@
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>44334.518068888894</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="I4" s="4">
+        <v>34405.0</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1.515864375E10</v>
+      </c>
+      <c r="M4" s="2">
+        <v>2.70229289E8</v>
+      </c>
+      <c r="N4" s="4">
+        <v>41342.0</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="T4" s="2">
+        <v>2.721517E7</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="V4" s="2">
+        <v>2.4998766749E10</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z4" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="AA4" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="AB4" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="AC4" s="2">
+        <v>2.721517E7</v>
+      </c>
+      <c r="AD4" s="2">
+        <v>2.4998448202E10</v>
+      </c>
+      <c r="AE4" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="AF4" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="AG4" s="4">
+        <v>43177.0</v>
+      </c>
+      <c r="AH4" s="4">
+        <v>43965.0</v>
+      </c>
+      <c r="AI4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="AJ4" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="AK4" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="AL4" s="4">
+        <v>41351.0</v>
+      </c>
+      <c r="AM4" s="4">
+        <v>43091.0</v>
+      </c>
+      <c r="AN4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="AO4" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="AP4" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ4" s="4">
+        <v>39874.0</v>
+      </c>
+      <c r="AR4" s="4">
+        <v>41527.0</v>
+      </c>
+      <c r="AS4" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="AX4" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="AY4" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="AZ4" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="BA4" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="BC4" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="BD4" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="BE4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="BF4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="BG4" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="BQ4" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="CO4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="CP4" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="CQ4" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="CR4" s="4">
+        <v>43598.0</v>
+      </c>
+      <c r="CS4" s="4">
+        <v>43626.0</v>
+      </c>
+      <c r="CT4" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="DI4" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="DJ4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="DK4" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="DL4" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="DM4" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="DN4" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="DO4" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="DP4" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="DQ4" s="7" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1h66cbUGy55OyDA-DH5yFT0ZNjRLK4dS9","Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf")</f>
+        <v>Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf</v>
+      </c>
+      <c r="DR4" s="7" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1798015fc46d86da","Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br")</f>
+        <v>Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
     <hyperlink r:id="rId2" ref="DO3"/>
     <hyperlink r:id="rId3" ref="DP3"/>
+    <hyperlink r:id="rId4" ref="DO4"/>
+    <hyperlink r:id="rId5" ref="DP4"/>
   </hyperlinks>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-05-18 19:01:40 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
+++ b/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="238">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -340,7 +340,7 @@
     <t>Deseja solicitar bolsa?</t>
   </si>
   <si>
-    <t>IES da última titulação</t>
+    <t>'IES da última titulação</t>
   </si>
   <si>
     <t>Quais as suas expectativas em relação ao curso?</t>
@@ -355,6 +355,18 @@
     <t>Upload do projeto</t>
   </si>
   <si>
+    <t>Foto para identificação</t>
+  </si>
+  <si>
+    <t>Nome do banco</t>
+  </si>
+  <si>
+    <t>Agência</t>
+  </si>
+  <si>
+    <t>Conta corrente</t>
+  </si>
+  <si>
     <t>[Document Studio] File Link</t>
   </si>
   <si>
@@ -635,6 +647,84 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1h66cbUGy55OyDA-DH5yFT0ZNjRLK4dS9</t>
+  </si>
+  <si>
+    <t>Mestrado em Engenharia Metalúrgica</t>
+  </si>
+  <si>
+    <t>Estágio à Docência</t>
+  </si>
+  <si>
+    <t>Desejo continuar a trabalhar com pesquisa de materiais metálicos e obter o título de doutora para dar início à docência.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1m3i5n421RNg5P5p9oasTq5UygvhJ84Yn</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=16xe1X-KLk-gWSaWSi0tuT4QGqQZZ6Nvh</t>
+  </si>
+  <si>
+    <t>Luiz T. F. Eleno</t>
+  </si>
+  <si>
+    <t>asdfgwqfwgv</t>
+  </si>
+  <si>
+    <t>eefgvwe</t>
+  </si>
+  <si>
+    <t>2ewvwefgvw</t>
+  </si>
+  <si>
+    <t>jkfgvjkvhjh</t>
+  </si>
+  <si>
+    <t>jhjhg</t>
+  </si>
+  <si>
+    <t>jkvkjgvkjvjkgv</t>
+  </si>
+  <si>
+    <t>j gjkgv jkgg jkgh</t>
+  </si>
+  <si>
+    <t>jghkjgh</t>
+  </si>
+  <si>
+    <t>kjg</t>
+  </si>
+  <si>
+    <t>gvjgjv</t>
+  </si>
+  <si>
+    <t>jvhjgv</t>
+  </si>
+  <si>
+    <t>inglês</t>
+  </si>
+  <si>
+    <t>jlklj</t>
+  </si>
+  <si>
+    <t>lnasdflçjkasv slgjsçkl</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1bzozzOUIHD7qP3GaB06IfN2h8s3qPqL0</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1pqdPC8jnM1pAL9H2SX-xcK7jPYV80v6j</t>
+  </si>
+  <si>
+    <t>jkbhkljb</t>
+  </si>
+  <si>
+    <t>0897089</t>
+  </si>
+  <si>
+    <t>0897089-0</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1CktcMLnlGhvcvjTV62f6O9r6PjuRf6F7</t>
   </si>
 </sst>
 </file>
@@ -644,7 +734,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy h:mm:ss"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -654,6 +744,7 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -677,12 +768,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -694,10 +788,13 @@
     <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -911,7 +1008,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="125" width="21.57"/>
+    <col customWidth="1" min="1" max="129" width="21.57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1257,7 +1354,7 @@
       <c r="DJ1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="DK1" s="1" t="s">
+      <c r="DK1" s="3" t="s">
         <v>109</v>
       </c>
       <c r="DL1" s="1" t="s">
@@ -1272,49 +1369,61 @@
       <c r="DO1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="DP1" s="2" t="s">
+      <c r="DP1" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="DQ1" s="2" t="s">
+      <c r="DQ1" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="DR1" s="2" t="s">
+      <c r="DR1" s="3" t="s">
         <v>116</v>
+      </c>
+      <c r="DS1" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="DT1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="DU1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="DV1" s="2" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="4">
         <v>44302.574963900464</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H2" s="2">
         <v>0.0</v>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="5">
         <v>28034.0</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="L2" s="2">
         <v>2.3542135423423E13</v>
@@ -1322,253 +1431,257 @@
       <c r="M2" s="2">
         <v>2.5425423413341E13</v>
       </c>
-      <c r="N2" s="4">
+      <c r="N2" s="5">
         <v>36892.0</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="P2" s="2">
         <v>1176388.0</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="T2" s="2">
         <v>1.260634E7</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="V2" s="2">
         <v>1.230362333E9</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="AC2" s="5" t="s">
-        <v>134</v>
+        <v>128</v>
+      </c>
+      <c r="AC2" s="6" t="s">
+        <v>138</v>
       </c>
       <c r="AD2" s="2">
         <v>1.1023434413E10</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="AG2" s="4">
+        <v>140</v>
+      </c>
+      <c r="AG2" s="5">
         <v>41183.0</v>
       </c>
-      <c r="AH2" s="4">
+      <c r="AH2" s="5">
         <v>41763.0</v>
       </c>
       <c r="AI2" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="AJ2" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="AK2" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="AL2" s="4">
+        <v>142</v>
+      </c>
+      <c r="AL2" s="5">
         <v>40087.0</v>
       </c>
-      <c r="AM2" s="4">
+      <c r="AM2" s="5">
         <v>41000.0</v>
       </c>
       <c r="AN2" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="AO2" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="AP2" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AQ2" s="4">
+        <v>143</v>
+      </c>
+      <c r="AQ2" s="5">
         <v>36526.0</v>
       </c>
-      <c r="AR2" s="4">
+      <c r="AR2" s="5">
         <v>37288.0</v>
       </c>
       <c r="AS2" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="AX2" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="AY2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="AZ2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BA2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BB2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="BC2" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BD2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BE2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BF2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BG2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="BH2" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="BI2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BJ2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BK2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BL2" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="BQ2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="BR2" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="BS2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="BT2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BU2" s="5">
+        <v>41763.0</v>
+      </c>
+      <c r="BV2" s="5">
+        <v>42095.0</v>
+      </c>
+      <c r="BW2" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="CO2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="CP2" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="CQ2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="CR2" s="5">
+        <v>41763.0</v>
+      </c>
+      <c r="CS2" s="5">
+        <v>44337.0</v>
+      </c>
+      <c r="CT2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="CU2" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="AY2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="AZ2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BA2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BB2" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="BC2" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BE2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BF2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BG2" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="BH2" s="2" t="s">
+      <c r="CV2" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="CW2" s="5">
+        <v>41275.0</v>
+      </c>
+      <c r="CX2" s="5">
+        <v>41456.0</v>
+      </c>
+      <c r="CY2" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="BI2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="BJ2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="BK2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="BL2" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="BQ2" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="BR2" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BS2" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="BT2" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="BU2" s="4">
-        <v>41763.0</v>
-      </c>
-      <c r="BV2" s="4">
-        <v>42095.0</v>
-      </c>
-      <c r="BW2" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="CO2" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="CP2" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="CQ2" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="CR2" s="4">
-        <v>41763.0</v>
-      </c>
-      <c r="CS2" s="4">
-        <v>44337.0</v>
-      </c>
-      <c r="CT2" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="CU2" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="CV2" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="CW2" s="4">
-        <v>41275.0</v>
-      </c>
-      <c r="CX2" s="4">
-        <v>41456.0</v>
-      </c>
-      <c r="CY2" s="2" t="s">
-        <v>140</v>
-      </c>
       <c r="DI2" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="DJ2" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="DK2" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="DL2" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="DM2" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="DN2" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="DO2" s="6" t="s">
-        <v>154</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="DO2" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="DP2" s="8"/>
+      <c r="DQ2" s="8"/>
+      <c r="DR2" s="8"/>
+      <c r="DS2" s="8"/>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>44302.74436298611</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H3" s="2">
         <v>0.0</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="5">
         <v>28034.0</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="K3" s="2">
         <v>3.458072340857E12</v>
@@ -1579,7 +1692,7 @@
       <c r="M3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="N3" s="4">
+      <c r="N3" s="5">
         <v>36892.0</v>
       </c>
       <c r="O3" s="2">
@@ -1601,7 +1714,7 @@
         <v>3.458072340857E12</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="V3" s="2">
         <v>3.458072340857E12</v>
@@ -1636,14 +1749,14 @@
       <c r="AF3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="AG3" s="4">
+      <c r="AG3" s="5">
         <v>36892.0</v>
       </c>
-      <c r="AH3" s="4" t="s">
-        <v>157</v>
+      <c r="AH3" s="5" t="s">
+        <v>161</v>
       </c>
       <c r="AI3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="AJ3" s="2">
         <v>3.458072340857E12</v>
@@ -1651,14 +1764,14 @@
       <c r="AK3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="AL3" s="4">
+      <c r="AL3" s="5">
         <v>36892.0</v>
       </c>
-      <c r="AM3" s="4">
+      <c r="AM3" s="5">
         <v>36892.0</v>
       </c>
       <c r="AN3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="AO3" s="2">
         <v>3.458072340857E12</v>
@@ -1666,14 +1779,14 @@
       <c r="AP3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="AQ3" s="4">
+      <c r="AQ3" s="5">
         <v>36892.0</v>
       </c>
-      <c r="AR3" s="4">
+      <c r="AR3" s="5">
         <v>36892.0</v>
       </c>
       <c r="AS3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="AT3" s="2">
         <v>3.458072340857E12</v>
@@ -1681,258 +1794,262 @@
       <c r="AU3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="AV3" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="AW3" s="4">
+      <c r="AV3" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="AW3" s="5">
         <v>402560.0</v>
       </c>
       <c r="AX3" s="2">
         <v>3.458072340857E12</v>
       </c>
       <c r="AY3" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="AZ3" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="BA3" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="BB3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="BC3" s="2">
         <v>3.458072340857E12</v>
       </c>
       <c r="BD3" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="BE3" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="BF3" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="BG3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="BH3" s="2">
         <v>3.458072340857E12</v>
       </c>
       <c r="BI3" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="BJ3" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="BK3" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="BL3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="BM3" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="BN3" s="2" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="BO3" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="BP3" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="BQ3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="BR3" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="BS3" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="BT3" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="BU3" s="4">
+        <v>166</v>
+      </c>
+      <c r="BU3" s="5">
         <v>36892.0</v>
       </c>
-      <c r="BV3" s="4">
+      <c r="BV3" s="5">
         <v>37289.0</v>
       </c>
       <c r="BW3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="BX3" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="BY3" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="BZ3" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="CA3" s="4">
+        <v>152</v>
+      </c>
+      <c r="CA3" s="5">
         <v>37682.0</v>
       </c>
-      <c r="CB3" s="4">
+      <c r="CB3" s="5">
         <v>38080.0</v>
       </c>
       <c r="CC3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="CD3" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="CE3" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="CF3" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="CF3" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="CG3" s="4">
+      <c r="CG3" s="5">
         <v>41255.0</v>
       </c>
-      <c r="CH3" s="4">
+      <c r="CH3" s="5">
         <v>41591.0</v>
       </c>
       <c r="CI3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="CJ3" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="CK3" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="CL3" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="CM3" s="4">
+        <v>152</v>
+      </c>
+      <c r="CM3" s="5">
         <v>40065.0</v>
       </c>
-      <c r="CN3" s="4">
+      <c r="CN3" s="5">
         <v>44334.0</v>
       </c>
       <c r="CO3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="CP3" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="CQ3" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="CR3" s="4">
+        <v>174</v>
+      </c>
+      <c r="CR3" s="5">
         <v>37987.0</v>
       </c>
       <c r="CT3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="CU3" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="CV3" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="CW3" s="4">
+        <v>176</v>
+      </c>
+      <c r="CW3" s="5">
         <v>45111.0</v>
       </c>
       <c r="CY3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="CZ3" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="DA3" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="DB3" s="4">
+        <v>178</v>
+      </c>
+      <c r="DB3" s="5">
         <v>153862.0</v>
       </c>
-      <c r="DC3" s="4">
+      <c r="DC3" s="5">
         <v>4333.0</v>
       </c>
       <c r="DD3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="DE3" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="DF3" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="DG3" s="4" t="s">
-        <v>177</v>
+        <v>180</v>
+      </c>
+      <c r="DG3" s="5" t="s">
+        <v>181</v>
       </c>
       <c r="DI3" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="DJ3" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="DK3" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="DL3" s="2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="DM3" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="DN3" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="DO3" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="DP3" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="DQ3" s="7" t="str">
+        <v>184</v>
+      </c>
+      <c r="DO3" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="DP3" s="8"/>
+      <c r="DQ3" s="8"/>
+      <c r="DR3" s="8"/>
+      <c r="DS3" s="8"/>
+      <c r="DT3" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="DU3" s="9" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1NOr-z6RTE9-w0_Zl-yNqVx1YerdXTO4Q","Inscrição PPGEM EEL-USP - Elenão.pdf")</f>
         <v>Inscrição PPGEM EEL-USP - Elenão.pdf</v>
       </c>
-      <c r="DR3" s="7" t="str">
+      <c r="DV3" s="9" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/178dc74aa5270d67","Email sent to luizeleno@gmail.com, ppgem-eel@usp.br")</f>
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="4">
         <v>44334.518068888894</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="H4" s="2">
         <v>0.0</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="5">
         <v>34405.0</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="L4" s="2">
         <v>1.515864375E10</v>
@@ -1940,47 +2057,47 @@
       <c r="M4" s="2">
         <v>2.70229289E8</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4" s="5">
         <v>41342.0</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="R4" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="S4" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>188</v>
       </c>
       <c r="T4" s="2">
         <v>2.721517E7</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="V4" s="2">
         <v>2.4998766749E10</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="X4" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="Y4" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="Y4" s="2" t="s">
-        <v>191</v>
-      </c>
       <c r="Z4" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="AA4" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="AA4" s="2" t="s">
-        <v>188</v>
-      </c>
       <c r="AB4" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="AC4" s="2">
         <v>2.721517E7</v>
@@ -1989,142 +2106,526 @@
         <v>2.4998448202E10</v>
       </c>
       <c r="AE4" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="AF4" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="AG4" s="4">
+        <v>202</v>
+      </c>
+      <c r="AG4" s="5">
         <v>43177.0</v>
       </c>
-      <c r="AH4" s="4">
+      <c r="AH4" s="5">
         <v>43965.0</v>
       </c>
       <c r="AI4" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="AJ4" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="AK4" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="AL4" s="4">
+        <v>203</v>
+      </c>
+      <c r="AL4" s="5">
         <v>41351.0</v>
       </c>
-      <c r="AM4" s="4">
+      <c r="AM4" s="5">
         <v>43091.0</v>
       </c>
       <c r="AN4" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="AO4" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="AP4" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="AQ4" s="5">
+        <v>39874.0</v>
+      </c>
+      <c r="AR4" s="5">
+        <v>41527.0</v>
+      </c>
+      <c r="AS4" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="AX4" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="AY4" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="AZ4" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BA4" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BB4" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="BC4" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BD4" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BE4" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="BF4" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="BG4" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="BQ4" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="CO4" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="CP4" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="AQ4" s="4">
-        <v>39874.0</v>
-      </c>
-      <c r="AR4" s="4">
-        <v>41527.0</v>
-      </c>
-      <c r="AS4" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="AX4" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AY4" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="AZ4" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BA4" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BB4" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="BC4" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD4" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="BE4" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="BF4" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="BG4" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="BQ4" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="CO4" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="CP4" s="2" t="s">
-        <v>197</v>
-      </c>
       <c r="CQ4" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="CR4" s="4">
+        <v>206</v>
+      </c>
+      <c r="CR4" s="5">
         <v>43598.0</v>
       </c>
-      <c r="CS4" s="4">
+      <c r="CS4" s="5">
         <v>43626.0</v>
       </c>
       <c r="CT4" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="DI4" s="2" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="DJ4" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="DK4" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="DL4" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="DM4" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="DN4" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="DO4" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="DP4" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="DQ4" s="7" t="str">
+        <v>209</v>
+      </c>
+      <c r="DO4" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="DP4" s="8"/>
+      <c r="DQ4" s="8"/>
+      <c r="DR4" s="8"/>
+      <c r="DS4" s="8"/>
+      <c r="DT4" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="DU4" s="9" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1h66cbUGy55OyDA-DH5yFT0ZNjRLK4dS9","Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf")</f>
         <v>Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf</v>
       </c>
-      <c r="DR4" s="7" t="str">
+      <c r="DV4" s="9" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1798015fc46d86da","Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br")</f>
         <v>Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>44334.58987285879</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="I5" s="5">
+        <v>34405.0</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="L5" s="2">
+        <v>1.515864375E10</v>
+      </c>
+      <c r="M5" s="2">
+        <v>2.70229289E8</v>
+      </c>
+      <c r="N5" s="5">
+        <v>41342.0</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="T5" s="2">
+        <v>2.721517E7</v>
+      </c>
+      <c r="U5" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="V5" s="2">
+        <v>2.4998766749E10</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="Z5" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="AA5" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="AB5" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="AC5" s="2">
+        <v>2.721517E7</v>
+      </c>
+      <c r="AD5" s="2">
+        <v>2.4998448202E10</v>
+      </c>
+      <c r="AE5" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="AF5" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="AG5" s="5">
+        <v>43177.0</v>
+      </c>
+      <c r="AH5" s="5">
+        <v>43965.0</v>
+      </c>
+      <c r="AI5" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AJ5" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="AK5" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="AL5" s="5">
+        <v>41351.0</v>
+      </c>
+      <c r="AM5" s="5">
+        <v>43091.0</v>
+      </c>
+      <c r="AN5" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="AX5" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="AY5" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="AZ5" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BA5" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BB5" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="BC5" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BD5" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BE5" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="BF5" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="BG5" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="BQ5" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="CO5" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="CP5" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="CQ5" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="CR5" s="5">
+        <v>43598.0</v>
+      </c>
+      <c r="CS5" s="5">
+        <v>43626.0</v>
+      </c>
+      <c r="CT5" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="DI5" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="DJ5" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="DK5" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="DL5" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="DM5" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DN5" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="DO5" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="DP5" s="8"/>
+      <c r="DQ5" s="8"/>
+      <c r="DR5" s="8"/>
+      <c r="DS5" s="8"/>
+      <c r="DT5" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="DU5" s="9" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=16xe1X-KLk-gWSaWSi0tuT4QGqQZZ6Nvh","Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf")</f>
+        <v>Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf</v>
+      </c>
+      <c r="DV5" s="9" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1798074b83a4bfeb","Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br")</f>
+        <v>Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>44334.643705254624</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="I6" s="5">
+        <v>28034.0</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="L6" s="2">
+        <v>2.34564652E8</v>
+      </c>
+      <c r="M6" s="2">
+        <v>2.4678697E7</v>
+      </c>
+      <c r="N6" s="5">
+        <v>36892.0</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="P6" s="2">
+        <v>436732.0</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="T6" s="2">
+        <v>2.5234423E7</v>
+      </c>
+      <c r="U6" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="V6" s="2">
+        <v>7.8657906897E10</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="Z6" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="AA6" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="AB6" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="AC6" s="2">
+        <v>6.7976987E7</v>
+      </c>
+      <c r="AD6" s="2">
+        <v>96976.0</v>
+      </c>
+      <c r="AE6" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="AF6" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="AG6" s="5">
+        <v>36892.0</v>
+      </c>
+      <c r="AH6" s="5">
+        <v>37289.0</v>
+      </c>
+      <c r="AI6" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="AX6" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="AY6" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="AZ6" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA6" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BB6" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="BQ6" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="CO6" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="DI6" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="DJ6" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="DL6" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="DM6" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DN6" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="DO6" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="DP6" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="DQ6" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="DR6" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="DS6" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="DT6" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="DU6" s="9" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1CktcMLnlGhvcvjTV62f6O9r6PjuRf6F7","Inscrição DOUTORADO PPGEM EEL-USP - Luiz T. F. Eleno.pdf")</f>
+        <v>Inscrição DOUTORADO PPGEM EEL-USP - Luiz T. F. Eleno.pdf</v>
+      </c>
+      <c r="DV6" s="9" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/17980bb7840d91a2","Email sent to luizeleno@gmail.com, ppgem-eel@usp.br")</f>
+        <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
     <hyperlink r:id="rId2" ref="DO3"/>
-    <hyperlink r:id="rId3" ref="DP3"/>
+    <hyperlink r:id="rId3" ref="DT3"/>
     <hyperlink r:id="rId4" ref="DO4"/>
-    <hyperlink r:id="rId5" ref="DP4"/>
+    <hyperlink r:id="rId5" ref="DT4"/>
+    <hyperlink r:id="rId6" ref="DO5"/>
+    <hyperlink r:id="rId7" ref="DT5"/>
+    <hyperlink r:id="rId8" ref="DO6"/>
+    <hyperlink r:id="rId9" ref="DP6"/>
+    <hyperlink r:id="rId10" ref="DT6"/>
   </hyperlinks>
-  <drawing r:id="rId6"/>
+  <drawing r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-05-19 13:02:44 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
+++ b/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="243">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -725,6 +725,21 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1CktcMLnlGhvcvjTV62f6O9r6PjuRf6F7</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=13E4_KQgUhjW71iR3PKMMf3Kx2anvMT_z</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1kx0MGI4JobJo44RpwXTVgJDWmH4vp0vl</t>
+  </si>
+  <si>
+    <t>Banco do Brasil</t>
+  </si>
+  <si>
+    <t>02623</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1f8nNJpkKgKFm46Uhkr1E58gKe-IeKGS0</t>
   </si>
 </sst>
 </file>
@@ -2613,6 +2628,217 @@
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>44335.405438125</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="I7" s="5">
+        <v>34405.0</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="L7" s="2">
+        <v>1.515864375E10</v>
+      </c>
+      <c r="M7" s="2">
+        <v>2.70229289E8</v>
+      </c>
+      <c r="N7" s="5">
+        <v>41342.0</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="T7" s="2">
+        <v>2.721517E7</v>
+      </c>
+      <c r="U7" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="V7" s="2">
+        <v>2.4998766749E10</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="Z7" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="AA7" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="AB7" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="AC7" s="2">
+        <v>2.721517E7</v>
+      </c>
+      <c r="AD7" s="2">
+        <v>2.4998448202E10</v>
+      </c>
+      <c r="AE7" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="AF7" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="AG7" s="5">
+        <v>43177.0</v>
+      </c>
+      <c r="AH7" s="5">
+        <v>43965.0</v>
+      </c>
+      <c r="AI7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AJ7" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="AK7" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="AL7" s="5">
+        <v>41351.0</v>
+      </c>
+      <c r="AM7" s="5">
+        <v>43091.0</v>
+      </c>
+      <c r="AN7" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="AX7" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="AY7" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="AZ7" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BA7" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="BB7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="BC7" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BD7" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BE7" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="BF7" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="BG7" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="BQ7" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="CO7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="CP7" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="CQ7" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="CR7" s="5">
+        <v>43598.0</v>
+      </c>
+      <c r="CS7" s="5">
+        <v>43626.0</v>
+      </c>
+      <c r="CT7" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="DI7" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="DJ7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="DL7" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="DM7" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DN7" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="DO7" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="DP7" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="DQ7" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="DR7" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="DS7" s="2">
+        <v>762857.0</v>
+      </c>
+      <c r="DT7" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="DU7" s="9" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1f8nNJpkKgKFm46Uhkr1E58gKe-IeKGS0","Inscrição DOUTORADO PPGEM EEL-USP - Rafaela dos Santos Silva.pdf")</f>
+        <v>Inscrição DOUTORADO PPGEM EEL-USP - Rafaela dos Santos Silva.pdf</v>
+      </c>
+      <c r="DV7" s="9" t="str">
+        <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/17984a7ce0ad9635","Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br")</f>
+        <v>Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="DO2"/>
@@ -2625,7 +2851,10 @@
     <hyperlink r:id="rId8" ref="DO6"/>
     <hyperlink r:id="rId9" ref="DP6"/>
     <hyperlink r:id="rId10" ref="DT6"/>
+    <hyperlink r:id="rId11" ref="DO7"/>
+    <hyperlink r:id="rId12" ref="DP7"/>
+    <hyperlink r:id="rId13" ref="DT7"/>
   </hyperlinks>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2021-06-30 13:00:36 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
+++ b/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
@@ -4,14 +4,76 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Respostas" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Document Studio Logs" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment authorId="0" ref="DW1">
+      <text>
+        <t xml:space="preserve">For workflow #form_890025668
+Respostas (Google Form)
+Created by luizeleno@usp.br on 2021-06-29 17:45</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="DX1">
+      <text>
+        <t xml:space="preserve">For workflow #form_890025668
+Respostas (Google Form)
+Created by luizeleno@usp.br on 2021-06-29 17:45</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="DY1">
+      <text>
+        <t xml:space="preserve">For workflow #form_890025668
+Respostas (Google Form)
+Created by luizeleno@usp.br on 2021-06-29 17:45</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="DT8">
+      <text>
+        <t xml:space="preserve">Updated on 2021-06-29 17:46 by luizeleno@usp.br</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="DU8">
+      <text>
+        <t xml:space="preserve">Updated on 2021-06-29 17:46 by luizeleno@usp.br</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="DV8">
+      <text>
+        <t xml:space="preserve">Updated on 2021-06-29 17:46 by luizeleno@usp.br</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="DW8">
+      <text>
+        <t xml:space="preserve">Updated on 2021-06-29 17:45 by luizeleno@usp.br</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="DX8">
+      <text>
+        <t xml:space="preserve">Updated on 2021-06-29 17:45 by luizeleno@usp.br</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="DY8">
+      <text>
+        <t xml:space="preserve">Updated on 2021-06-29 17:45 by luizeleno@usp.br</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="275">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -376,6 +438,15 @@
     <t>[Document Studio] Email Status</t>
   </si>
   <si>
+    <t>Response ID</t>
+  </si>
+  <si>
+    <t>Response Edit URL</t>
+  </si>
+  <si>
+    <t>Response Timestamp</t>
+  </si>
+  <si>
     <t>Luiz Eleno</t>
   </si>
   <si>
@@ -740,6 +811,93 @@
   </si>
   <si>
     <t>https://drive.google.com/open?id=1f8nNJpkKgKFm46Uhkr1E58gKe-IeKGS0</t>
+  </si>
+  <si>
+    <t>Erica Marcelino Freitas de Souza Silva</t>
+  </si>
+  <si>
+    <t>ericauffmetal@gmail.com</t>
+  </si>
+  <si>
+    <t>Negra</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>Angra dos Reis</t>
+  </si>
+  <si>
+    <t>Avenida Joaquim Leite, 380-APTO 706</t>
+  </si>
+  <si>
+    <t>Centro</t>
+  </si>
+  <si>
+    <t>Barra Mansa</t>
+  </si>
+  <si>
+    <t>Wagner de Oliveira Silva</t>
+  </si>
+  <si>
+    <t>Marido</t>
+  </si>
+  <si>
+    <t>Avenida Joaquim Leite 380</t>
+  </si>
+  <si>
+    <t>Universidade Federal Fluminense-UFF</t>
+  </si>
+  <si>
+    <t>Mestre em Engenharia Metalúrgica</t>
+  </si>
+  <si>
+    <t>Centro Universitário de Volta Redonda-UniFOA</t>
+  </si>
+  <si>
+    <t>Engenheira Mecânica</t>
+  </si>
+  <si>
+    <t>Estágio em Docência 1</t>
+  </si>
+  <si>
+    <t>A começar pela grande admiração que tenho por esta instituição, minhas expectativas são adquirir o melhor conhecimento possível, contribuir para o avanço da ciência e tecnologia e agregar valores ao programa.</t>
+  </si>
+  <si>
+    <t>Estudo da  microestrutura e do crescimento de trincas por corrosão-fadiga em cordões de solda obtidos pelos processos TIG e Laser no aço inoxidável austenítico 316L</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=15-3nbSQjtIYLoiipPj7MxXHFtt7aS2uT</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1h9-O89BRBr3S0Vt0R3E5m7Fc36gffeqp</t>
+  </si>
+  <si>
+    <t>0001</t>
+  </si>
+  <si>
+    <t>sim</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1QRgVJRloYrt01rUxubr6KIx72DAMv3mR</t>
+  </si>
+  <si>
+    <t>Email sent to ppgem-eel@usp.br, ericauffmetal@gmail.com</t>
+  </si>
+  <si>
+    <t>2_ABaOnueCPAePq-t4LWTCX-HNcICHdiDsvid9GLifyte_NLhi4V0qPTTHSLQSAA5euqvbqu4</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/forms/d/e/1FAIpQLSdcC8OxBYiJiDWMko1G13-gQfcteiPPgMJQaQNzpi9SQLUpvw/viewform?edit2=2_ABaOnueCPAePq-t4LWTCX-HNcICHdiDsvid9GLifyte_NLhi4V0qPTTHSLQSAA5euqvbqu4</t>
+  </si>
+  <si>
+    <t>Document Studio Logs</t>
+  </si>
+  <si>
+    <t>👋🏻 Please do not edit or delete this sheet)</t>
+  </si>
+  <si>
+    <t>ℹ️  Form row #8 in sheet "Respostas", run as luizeleno@usp.br (6547558433841371775), processed in 37 seconds.</t>
   </si>
 </sst>
 </file>
@@ -749,7 +907,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy h:mm:ss"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -759,7 +917,6 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
@@ -769,12 +926,30 @@
       <color rgb="FF0000FF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9DAF8"/>
+        <bgColor rgb="FFC9DAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0E0E3"/>
+        <bgColor rgb="FFD0E0E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor rgb="FFF4CCCC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -783,7 +958,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -791,8 +966,14 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
@@ -803,13 +984,13 @@
     <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -819,6 +1000,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1369,7 +1554,7 @@
       <c r="DJ1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="DK1" s="3" t="s">
+      <c r="DK1" s="2" t="s">
         <v>109</v>
       </c>
       <c r="DL1" s="1" t="s">
@@ -1384,16 +1569,16 @@
       <c r="DO1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="DP1" s="3" t="s">
+      <c r="DP1" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="DQ1" s="3" t="s">
+      <c r="DQ1" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="DR1" s="3" t="s">
+      <c r="DR1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="DS1" s="3" t="s">
+      <c r="DS1" s="2" t="s">
         <v>117</v>
       </c>
       <c r="DT1" s="2" t="s">
@@ -1405,40 +1590,49 @@
       <c r="DV1" s="2" t="s">
         <v>120</v>
       </c>
+      <c r="DW1" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="DX1" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="DY1" s="5" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="6">
         <v>44302.574963900464</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H2" s="2">
         <v>0.0</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="7">
         <v>28034.0</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="L2" s="2">
         <v>2.3542135423423E13</v>
@@ -1446,257 +1640,257 @@
       <c r="M2" s="2">
         <v>2.5425423413341E13</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="7">
         <v>36892.0</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="P2" s="2">
         <v>1176388.0</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="T2" s="2">
         <v>1.260634E7</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="V2" s="2">
         <v>1.230362333E9</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="AC2" s="6" t="s">
-        <v>138</v>
+        <v>131</v>
+      </c>
+      <c r="AC2" s="8" t="s">
+        <v>141</v>
       </c>
       <c r="AD2" s="2">
         <v>1.1023434413E10</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="AG2" s="5">
+        <v>143</v>
+      </c>
+      <c r="AG2" s="7">
         <v>41183.0</v>
       </c>
-      <c r="AH2" s="5">
+      <c r="AH2" s="7">
         <v>41763.0</v>
       </c>
       <c r="AI2" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AJ2" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="AK2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="AL2" s="5">
+        <v>145</v>
+      </c>
+      <c r="AL2" s="7">
         <v>40087.0</v>
       </c>
-      <c r="AM2" s="5">
+      <c r="AM2" s="7">
         <v>41000.0</v>
       </c>
       <c r="AN2" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AO2" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="AP2" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="AQ2" s="5">
+        <v>146</v>
+      </c>
+      <c r="AQ2" s="7">
         <v>36526.0</v>
       </c>
-      <c r="AR2" s="5">
+      <c r="AR2" s="7">
         <v>37288.0</v>
       </c>
       <c r="AS2" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="AX2" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="AY2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="BC2" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="BD2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BE2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BF2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BG2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="BH2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="BI2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BJ2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BK2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BL2" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BQ2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR2" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="BS2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="BT2" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="BU2" s="7">
+        <v>41763.0</v>
+      </c>
+      <c r="BV2" s="7">
+        <v>42095.0</v>
+      </c>
+      <c r="BW2" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="CO2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CP2" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="CQ2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="CR2" s="7">
+        <v>41763.0</v>
+      </c>
+      <c r="CS2" s="7">
+        <v>44337.0</v>
+      </c>
+      <c r="CT2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU2" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="AX2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="AY2" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="AZ2" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BA2" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BB2" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="BC2" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="BD2" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BE2" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BF2" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BG2" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="BH2" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="BI2" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="BJ2" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="BK2" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="BL2" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="BQ2" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="BR2" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="BS2" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="BT2" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="BU2" s="5">
-        <v>41763.0</v>
-      </c>
-      <c r="BV2" s="5">
-        <v>42095.0</v>
-      </c>
-      <c r="BW2" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="CO2" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="CP2" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="CQ2" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="CR2" s="5">
-        <v>41763.0</v>
-      </c>
-      <c r="CS2" s="5">
-        <v>44337.0</v>
-      </c>
-      <c r="CT2" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="CU2" s="2" t="s">
-        <v>141</v>
-      </c>
       <c r="CV2" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="CW2" s="5">
+        <v>156</v>
+      </c>
+      <c r="CW2" s="7">
         <v>41275.0</v>
       </c>
-      <c r="CX2" s="5">
+      <c r="CX2" s="7">
         <v>41456.0</v>
       </c>
       <c r="CY2" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="DI2" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="DJ2" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="DK2" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="DL2" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="DM2" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="DN2" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="DO2" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="DP2" s="8"/>
-      <c r="DQ2" s="8"/>
-      <c r="DR2" s="8"/>
-      <c r="DS2" s="8"/>
+        <v>160</v>
+      </c>
+      <c r="DO2" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="DP2" s="10"/>
+      <c r="DQ2" s="10"/>
+      <c r="DR2" s="10"/>
+      <c r="DS2" s="10"/>
     </row>
     <row r="3">
-      <c r="A3" s="4">
+      <c r="A3" s="6">
         <v>44302.74436298611</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H3" s="2">
         <v>0.0</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="7">
         <v>28034.0</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="K3" s="2">
         <v>3.458072340857E12</v>
@@ -1707,7 +1901,7 @@
       <c r="M3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="7">
         <v>36892.0</v>
       </c>
       <c r="O3" s="2">
@@ -1729,7 +1923,7 @@
         <v>3.458072340857E12</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="V3" s="2">
         <v>3.458072340857E12</v>
@@ -1764,14 +1958,14 @@
       <c r="AF3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="AG3" s="5">
+      <c r="AG3" s="7">
         <v>36892.0</v>
       </c>
-      <c r="AH3" s="5" t="s">
-        <v>161</v>
+      <c r="AH3" s="7" t="s">
+        <v>164</v>
       </c>
       <c r="AI3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AJ3" s="2">
         <v>3.458072340857E12</v>
@@ -1779,14 +1973,14 @@
       <c r="AK3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="AL3" s="5">
+      <c r="AL3" s="7">
         <v>36892.0</v>
       </c>
-      <c r="AM3" s="5">
+      <c r="AM3" s="7">
         <v>36892.0</v>
       </c>
       <c r="AN3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AO3" s="2">
         <v>3.458072340857E12</v>
@@ -1794,14 +1988,14 @@
       <c r="AP3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="AQ3" s="5">
+      <c r="AQ3" s="7">
         <v>36892.0</v>
       </c>
-      <c r="AR3" s="5">
+      <c r="AR3" s="7">
         <v>36892.0</v>
       </c>
       <c r="AS3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AT3" s="2">
         <v>3.458072340857E12</v>
@@ -1809,262 +2003,262 @@
       <c r="AU3" s="2">
         <v>3.458072340857E12</v>
       </c>
-      <c r="AV3" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="AW3" s="5">
+      <c r="AV3" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="AW3" s="7">
         <v>402560.0</v>
       </c>
       <c r="AX3" s="2">
         <v>3.458072340857E12</v>
       </c>
       <c r="AY3" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="AZ3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BA3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="BA3" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="BB3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="BC3" s="2">
         <v>3.458072340857E12</v>
       </c>
       <c r="BD3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BE3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="BE3" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="BF3" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BG3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="BH3" s="2">
         <v>3.458072340857E12</v>
       </c>
       <c r="BI3" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="BJ3" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BK3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BL3" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM3" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="BN3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="BL3" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="BM3" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="BN3" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="BO3" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="BP3" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BQ3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="BR3" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="BS3" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="BT3" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="BU3" s="5">
+        <v>169</v>
+      </c>
+      <c r="BU3" s="7">
         <v>36892.0</v>
       </c>
-      <c r="BV3" s="5">
+      <c r="BV3" s="7">
         <v>37289.0</v>
       </c>
       <c r="BW3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="BX3" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="BY3" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="BZ3" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="CA3" s="5">
+        <v>155</v>
+      </c>
+      <c r="CA3" s="7">
         <v>37682.0</v>
       </c>
-      <c r="CB3" s="5">
+      <c r="CB3" s="7">
         <v>38080.0</v>
       </c>
       <c r="CC3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="CD3" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="CE3" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="CF3" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="CE3" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="CF3" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="CG3" s="5">
+      <c r="CG3" s="7">
         <v>41255.0</v>
       </c>
-      <c r="CH3" s="5">
+      <c r="CH3" s="7">
         <v>41591.0</v>
       </c>
       <c r="CI3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="CJ3" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="CK3" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="CL3" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="CM3" s="5">
+        <v>155</v>
+      </c>
+      <c r="CM3" s="7">
         <v>40065.0</v>
       </c>
-      <c r="CN3" s="5">
+      <c r="CN3" s="7">
         <v>44334.0</v>
       </c>
       <c r="CO3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="CP3" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="CQ3" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="CR3" s="5">
+        <v>177</v>
+      </c>
+      <c r="CR3" s="7">
         <v>37987.0</v>
       </c>
       <c r="CT3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="CU3" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="CV3" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="CW3" s="5">
+        <v>179</v>
+      </c>
+      <c r="CW3" s="7">
         <v>45111.0</v>
       </c>
       <c r="CY3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="CZ3" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="DA3" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="DB3" s="5">
+        <v>181</v>
+      </c>
+      <c r="DB3" s="7">
         <v>153862.0</v>
       </c>
-      <c r="DC3" s="5">
+      <c r="DC3" s="7">
         <v>4333.0</v>
       </c>
       <c r="DD3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="DE3" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="DF3" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="DG3" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
+      </c>
+      <c r="DG3" s="7" t="s">
+        <v>184</v>
       </c>
       <c r="DI3" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="DJ3" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="DK3" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="DL3" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="DM3" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="DN3" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="DO3" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="DP3" s="8"/>
-      <c r="DQ3" s="8"/>
-      <c r="DR3" s="8"/>
-      <c r="DS3" s="8"/>
-      <c r="DT3" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="DU3" s="9" t="str">
+        <v>187</v>
+      </c>
+      <c r="DO3" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="DP3" s="10"/>
+      <c r="DQ3" s="10"/>
+      <c r="DR3" s="10"/>
+      <c r="DS3" s="10"/>
+      <c r="DT3" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="DU3" s="11" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1NOr-z6RTE9-w0_Zl-yNqVx1YerdXTO4Q","Inscrição PPGEM EEL-USP - Elenão.pdf")</f>
         <v>Inscrição PPGEM EEL-USP - Elenão.pdf</v>
       </c>
-      <c r="DV3" s="9" t="str">
+      <c r="DV3" s="11" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/178dc74aa5270d67","Email sent to luizeleno@gmail.com, ppgem-eel@usp.br")</f>
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="6">
         <v>44334.518068888894</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="H4" s="2">
         <v>0.0</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="7">
         <v>34405.0</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="L4" s="2">
         <v>1.515864375E10</v>
@@ -2072,47 +2266,47 @@
       <c r="M4" s="2">
         <v>2.70229289E8</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="7">
         <v>41342.0</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="Q4" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="S4" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="R4" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>192</v>
       </c>
       <c r="T4" s="2">
         <v>2.721517E7</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="V4" s="2">
         <v>2.4998766749E10</v>
       </c>
       <c r="W4" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="Y4" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="X4" s="2" t="s">
+      <c r="Z4" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="Y4" s="2" t="s">
+      <c r="AA4" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="Z4" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="AA4" s="2" t="s">
-        <v>192</v>
-      </c>
       <c r="AB4" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="AC4" s="2">
         <v>2.721517E7</v>
@@ -2121,171 +2315,171 @@
         <v>2.4998448202E10</v>
       </c>
       <c r="AE4" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AF4" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="AG4" s="5">
+        <v>205</v>
+      </c>
+      <c r="AG4" s="7">
         <v>43177.0</v>
       </c>
-      <c r="AH4" s="5">
+      <c r="AH4" s="7">
         <v>43965.0</v>
       </c>
       <c r="AI4" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AJ4" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AK4" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="AL4" s="5">
+        <v>206</v>
+      </c>
+      <c r="AL4" s="7">
         <v>41351.0</v>
       </c>
-      <c r="AM4" s="5">
+      <c r="AM4" s="7">
         <v>43091.0</v>
       </c>
       <c r="AN4" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AO4" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="AP4" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="AQ4" s="7">
+        <v>39874.0</v>
+      </c>
+      <c r="AR4" s="7">
+        <v>41527.0</v>
+      </c>
+      <c r="AS4" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="AX4" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="AY4" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ4" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA4" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB4" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="BC4" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="BD4" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BE4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="BF4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="BG4" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BQ4" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="CO4" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CP4" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="AP4" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="AQ4" s="5">
-        <v>39874.0</v>
-      </c>
-      <c r="AR4" s="5">
-        <v>41527.0</v>
-      </c>
-      <c r="AS4" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="AX4" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="AY4" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="AZ4" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BA4" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BB4" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="BC4" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="BD4" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="BE4" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="BF4" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="BG4" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="BQ4" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="CO4" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="CP4" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="CQ4" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="CR4" s="5">
+        <v>209</v>
+      </c>
+      <c r="CR4" s="7">
         <v>43598.0</v>
       </c>
-      <c r="CS4" s="5">
+      <c r="CS4" s="7">
         <v>43626.0</v>
       </c>
       <c r="CT4" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="DI4" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="DJ4" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="DK4" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="DL4" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="DM4" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="DN4" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="DO4" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="DP4" s="8"/>
-      <c r="DQ4" s="8"/>
-      <c r="DR4" s="8"/>
-      <c r="DS4" s="8"/>
-      <c r="DT4" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="DU4" s="9" t="str">
+        <v>212</v>
+      </c>
+      <c r="DO4" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="DP4" s="10"/>
+      <c r="DQ4" s="10"/>
+      <c r="DR4" s="10"/>
+      <c r="DS4" s="10"/>
+      <c r="DT4" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="DU4" s="11" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1h66cbUGy55OyDA-DH5yFT0ZNjRLK4dS9","Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf")</f>
         <v>Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf</v>
       </c>
-      <c r="DV4" s="9" t="str">
+      <c r="DV4" s="11" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1798015fc46d86da","Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br")</f>
         <v>Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4">
+      <c r="A5" s="6">
         <v>44334.58987285879</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="H5" s="2">
         <v>0.0</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="7">
         <v>34405.0</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="L5" s="2">
         <v>1.515864375E10</v>
@@ -2293,47 +2487,47 @@
       <c r="M5" s="2">
         <v>2.70229289E8</v>
       </c>
-      <c r="N5" s="5">
+      <c r="N5" s="7">
         <v>41342.0</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="Q5" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="S5" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>192</v>
       </c>
       <c r="T5" s="2">
         <v>2.721517E7</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="V5" s="2">
         <v>2.4998766749E10</v>
       </c>
       <c r="W5" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="Y5" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="X5" s="2" t="s">
+      <c r="Z5" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="Y5" s="2" t="s">
+      <c r="AA5" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="Z5" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="AA5" s="2" t="s">
-        <v>192</v>
-      </c>
       <c r="AB5" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="AC5" s="2">
         <v>2.721517E7</v>
@@ -2342,156 +2536,156 @@
         <v>2.4998448202E10</v>
       </c>
       <c r="AE5" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AF5" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="AG5" s="7">
+        <v>43177.0</v>
+      </c>
+      <c r="AH5" s="7">
+        <v>43965.0</v>
+      </c>
+      <c r="AI5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ5" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="AK5" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="AL5" s="7">
+        <v>41351.0</v>
+      </c>
+      <c r="AM5" s="7">
+        <v>43091.0</v>
+      </c>
+      <c r="AN5" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="AX5" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="AY5" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ5" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA5" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="BC5" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="BD5" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BE5" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="BF5" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="BG5" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BQ5" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="CO5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CP5" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="CQ5" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="CR5" s="7">
+        <v>43598.0</v>
+      </c>
+      <c r="CS5" s="7">
+        <v>43626.0</v>
+      </c>
+      <c r="CT5" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="DI5" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="DJ5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="DK5" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="DL5" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="DM5" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="DN5" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="AG5" s="5">
-        <v>43177.0</v>
-      </c>
-      <c r="AH5" s="5">
-        <v>43965.0</v>
-      </c>
-      <c r="AI5" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="AJ5" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="AK5" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="AL5" s="5">
-        <v>41351.0</v>
-      </c>
-      <c r="AM5" s="5">
-        <v>43091.0</v>
-      </c>
-      <c r="AN5" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="AX5" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="AY5" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="AZ5" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BA5" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BB5" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="BC5" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="BD5" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="BE5" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="BF5" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="BG5" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="BQ5" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="CO5" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="CP5" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="CQ5" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="CR5" s="5">
-        <v>43598.0</v>
-      </c>
-      <c r="CS5" s="5">
-        <v>43626.0</v>
-      </c>
-      <c r="CT5" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="DI5" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="DJ5" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="DK5" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="DL5" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="DM5" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="DN5" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="DO5" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="DP5" s="8"/>
-      <c r="DQ5" s="8"/>
-      <c r="DR5" s="8"/>
-      <c r="DS5" s="8"/>
-      <c r="DT5" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="DU5" s="9" t="str">
+      <c r="DO5" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="DP5" s="10"/>
+      <c r="DQ5" s="10"/>
+      <c r="DR5" s="10"/>
+      <c r="DS5" s="10"/>
+      <c r="DT5" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="DU5" s="11" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=16xe1X-KLk-gWSaWSi0tuT4QGqQZZ6Nvh","Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf")</f>
         <v>Inscrição PPGEM EEL-USP - Rafaela dos Santos Silva.pdf</v>
       </c>
-      <c r="DV5" s="9" t="str">
+      <c r="DV5" s="11" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/1798074b83a4bfeb","Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br")</f>
         <v>Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4">
+      <c r="A6" s="6">
         <v>44334.643705254624</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H6" s="2">
         <v>0.0</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="7">
         <v>28034.0</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="L6" s="2">
         <v>2.34564652E8</v>
@@ -2499,50 +2693,50 @@
       <c r="M6" s="2">
         <v>2.4678697E7</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6" s="7">
         <v>36892.0</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="P6" s="2">
         <v>436732.0</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="T6" s="2">
         <v>2.5234423E7</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="V6" s="2">
         <v>7.8657906897E10</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="Z6" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="AB6" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="AC6" s="2">
         <v>6.7976987E7</v>
@@ -2551,116 +2745,116 @@
         <v>96976.0</v>
       </c>
       <c r="AE6" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="AF6" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="AG6" s="5">
+        <v>231</v>
+      </c>
+      <c r="AG6" s="7">
         <v>36892.0</v>
       </c>
-      <c r="AH6" s="5">
+      <c r="AH6" s="7">
         <v>37289.0</v>
       </c>
       <c r="AI6" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="AX6" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="AY6" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="AZ6" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BA6" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="BA6" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="BB6" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="BQ6" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="CO6" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="DI6" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="DJ6" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="DL6" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="DM6" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="DN6" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="DO6" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="DP6" s="7" t="s">
-        <v>233</v>
+        <v>234</v>
+      </c>
+      <c r="DO6" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="DP6" s="9" t="s">
+        <v>236</v>
       </c>
       <c r="DQ6" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="DR6" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
+      </c>
+      <c r="DR6" s="8" t="s">
+        <v>238</v>
       </c>
       <c r="DS6" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="DT6" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="DU6" s="9" t="str">
+        <v>239</v>
+      </c>
+      <c r="DT6" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="DU6" s="11" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1CktcMLnlGhvcvjTV62f6O9r6PjuRf6F7","Inscrição DOUTORADO PPGEM EEL-USP - Luiz T. F. Eleno.pdf")</f>
         <v>Inscrição DOUTORADO PPGEM EEL-USP - Luiz T. F. Eleno.pdf</v>
       </c>
-      <c r="DV6" s="9" t="str">
+      <c r="DV6" s="11" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/17980bb7840d91a2","Email sent to luizeleno@gmail.com, ppgem-eel@usp.br")</f>
         <v>Email sent to luizeleno@gmail.com, ppgem-eel@usp.br</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4">
+      <c r="A7" s="6">
         <v>44335.405438125</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="H7" s="2">
         <v>0.0</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="7">
         <v>34405.0</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="L7" s="2">
         <v>1.515864375E10</v>
@@ -2668,47 +2862,47 @@
       <c r="M7" s="2">
         <v>2.70229289E8</v>
       </c>
-      <c r="N7" s="5">
+      <c r="N7" s="7">
         <v>41342.0</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="Q7" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="S7" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>192</v>
       </c>
       <c r="T7" s="2">
         <v>2.721517E7</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="V7" s="2">
         <v>2.4998766749E10</v>
       </c>
       <c r="W7" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="Y7" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="X7" s="2" t="s">
+      <c r="Z7" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="Y7" s="2" t="s">
+      <c r="AA7" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="Z7" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="AA7" s="2" t="s">
-        <v>192</v>
-      </c>
       <c r="AB7" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="AC7" s="2">
         <v>2.721517E7</v>
@@ -2717,144 +2911,402 @@
         <v>2.4998448202E10</v>
       </c>
       <c r="AE7" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AF7" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="AG7" s="7">
+        <v>43177.0</v>
+      </c>
+      <c r="AH7" s="7">
+        <v>43965.0</v>
+      </c>
+      <c r="AI7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ7" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="AK7" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="AL7" s="7">
+        <v>41351.0</v>
+      </c>
+      <c r="AM7" s="7">
+        <v>43091.0</v>
+      </c>
+      <c r="AN7" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="AX7" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="AY7" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ7" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA7" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="BC7" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="BD7" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="BE7" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="BF7" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="BG7" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BQ7" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="CO7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CP7" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="CQ7" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="CR7" s="7">
+        <v>43598.0</v>
+      </c>
+      <c r="CS7" s="7">
+        <v>43626.0</v>
+      </c>
+      <c r="CT7" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="DI7" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="DJ7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="DL7" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="DM7" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="DN7" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="AG7" s="5">
-        <v>43177.0</v>
-      </c>
-      <c r="AH7" s="5">
-        <v>43965.0</v>
-      </c>
-      <c r="AI7" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="AJ7" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="AK7" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="AL7" s="5">
-        <v>41351.0</v>
-      </c>
-      <c r="AM7" s="5">
-        <v>43091.0</v>
-      </c>
-      <c r="AN7" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="AX7" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="AY7" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="AZ7" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BA7" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="BB7" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="BC7" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="BD7" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="BE7" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="BF7" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="BG7" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="BQ7" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="CO7" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="CP7" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="CQ7" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="CR7" s="5">
-        <v>43598.0</v>
-      </c>
-      <c r="CS7" s="5">
-        <v>43626.0</v>
-      </c>
-      <c r="CT7" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="DI7" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="DJ7" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="DL7" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="DM7" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="DN7" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="DO7" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="DP7" s="7" t="s">
-        <v>239</v>
+      <c r="DO7" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="DP7" s="9" t="s">
+        <v>242</v>
       </c>
       <c r="DQ7" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="DR7" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
+      </c>
+      <c r="DR7" s="8" t="s">
+        <v>244</v>
       </c>
       <c r="DS7" s="2">
         <v>762857.0</v>
       </c>
-      <c r="DT7" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="DU7" s="9" t="str">
+      <c r="DT7" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="DU7" s="11" t="str">
         <f>HYPERLINK("https://drive.google.com/open?id=1f8nNJpkKgKFm46Uhkr1E58gKe-IeKGS0","Inscrição DOUTORADO PPGEM EEL-USP - Rafaela dos Santos Silva.pdf")</f>
         <v>Inscrição DOUTORADO PPGEM EEL-USP - Rafaela dos Santos Silva.pdf</v>
       </c>
-      <c r="DV7" s="9" t="str">
+      <c r="DV7" s="11" t="str">
         <f>HYPERLINK("https://mail.google.com/mail/u/?authuser=luizeleno@usp.br#all/17984a7ce0ad9635","Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br")</f>
         <v>Email sent to rafaelasantos@id.uff.br, ppgem-eel@usp.br</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6">
+        <v>44376.739958148144</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="I8" s="7">
+        <v>31187.0</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="L8" s="2">
+        <v>1.146228171E10</v>
+      </c>
+      <c r="M8" s="2">
+        <v>2.17138544E8</v>
+      </c>
+      <c r="N8" s="7">
+        <v>39863.0</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="P8" s="2">
+        <v>1.2500532E7</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="T8" s="2">
+        <v>2.7330043E7</v>
+      </c>
+      <c r="U8" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="V8" s="2">
+        <v>2.4999416211E10</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="Z8" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="AA8" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="AB8" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="AC8" s="2">
+        <v>2.7330043E7</v>
+      </c>
+      <c r="AD8" s="2">
+        <v>2.4992122038E10</v>
+      </c>
+      <c r="AE8" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="AF8" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="AG8" s="7">
+        <v>42982.0</v>
+      </c>
+      <c r="AH8" s="7">
+        <v>43903.0</v>
+      </c>
+      <c r="AI8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ8" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="AK8" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="AL8" s="7">
+        <v>40211.0</v>
+      </c>
+      <c r="AM8" s="7">
+        <v>42182.0</v>
+      </c>
+      <c r="AN8" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="AX8" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="AY8" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ8" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA8" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB8" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="BQ8" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="CO8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CP8" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="CQ8" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="CR8" s="7">
+        <v>43192.0</v>
+      </c>
+      <c r="CS8" s="7">
+        <v>43248.0</v>
+      </c>
+      <c r="CT8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU8" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="CV8" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="CW8" s="7">
+        <v>43395.0</v>
+      </c>
+      <c r="CX8" s="7">
+        <v>43454.0</v>
+      </c>
+      <c r="CY8" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="DI8" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="DJ8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="DL8" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="DM8" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="DN8" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="DO8" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="DP8" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="DQ8" s="2">
+        <v>5.4873606E7</v>
+      </c>
+      <c r="DR8" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="DS8" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="DT8" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="DU8" s="11" t="str">
+        <f>HYPERLINK("https://drive.google.com/open?id=1QRgVJRloYrt01rUxubr6KIx72DAMv3mR","Inscrição DOUTORADO PPGEM EEL-USP - Erica Marcelino Freitas de Souza Silva.pdf")</f>
+        <v>Inscrição DOUTORADO PPGEM EEL-USP - Erica Marcelino Freitas de Souza Silva.pdf</v>
+      </c>
+      <c r="DV8" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="DW8" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="DX8" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="DY8" s="7">
+        <v>44376.739958148144</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="DO2"/>
-    <hyperlink r:id="rId2" ref="DO3"/>
-    <hyperlink r:id="rId3" ref="DT3"/>
-    <hyperlink r:id="rId4" ref="DO4"/>
-    <hyperlink r:id="rId5" ref="DT4"/>
-    <hyperlink r:id="rId6" ref="DO5"/>
-    <hyperlink r:id="rId7" ref="DT5"/>
-    <hyperlink r:id="rId8" ref="DO6"/>
-    <hyperlink r:id="rId9" ref="DP6"/>
-    <hyperlink r:id="rId10" ref="DT6"/>
-    <hyperlink r:id="rId11" ref="DO7"/>
-    <hyperlink r:id="rId12" ref="DP7"/>
-    <hyperlink r:id="rId13" ref="DT7"/>
+    <hyperlink r:id="rId2" ref="DO2"/>
+    <hyperlink r:id="rId3" ref="DO3"/>
+    <hyperlink r:id="rId4" ref="DT3"/>
+    <hyperlink r:id="rId5" ref="DO4"/>
+    <hyperlink r:id="rId6" ref="DT4"/>
+    <hyperlink r:id="rId7" ref="DO5"/>
+    <hyperlink r:id="rId8" ref="DT5"/>
+    <hyperlink r:id="rId9" ref="DO6"/>
+    <hyperlink r:id="rId10" ref="DP6"/>
+    <hyperlink r:id="rId11" ref="DT6"/>
+    <hyperlink r:id="rId12" ref="DO7"/>
+    <hyperlink r:id="rId13" ref="DP7"/>
+    <hyperlink r:id="rId14" ref="DT7"/>
+    <hyperlink r:id="rId15" ref="DO8"/>
+    <hyperlink r:id="rId16" ref="DP8"/>
+    <hyperlink r:id="rId17" ref="DT8"/>
+    <hyperlink r:id="rId18" ref="DX8"/>
   </hyperlinks>
-  <drawing r:id="rId14"/>
+  <drawing r:id="rId19"/>
+  <legacyDrawing r:id="rId20"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6">
+        <v>44376.74002457176</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6">
+        <v>44376.74045414352</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build site at 2026-05-25 13:38:13 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
+++ b/_Drive/Formularios/Doutorado-FluxoContinuo/Inscrição para Doutorado (respostas).xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Respostas" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Document Studio Logs" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="Respostas" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Document Studio Logs" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -3294,6 +3294,10 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>